<commit_message>
Correct the MAINT record: UAT-01 is still open
The block was marked done, but its own criterion reads "every acceptance
criterion under MAINT is met" and UAT-01 is not: the interface has to be
evaluated by maintenance coordinators, which no amount of code closes.

MAINT is 7 of 8 subtasks, so Actual % moves 1.888 -> 2.203, not to 2.517.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SmartFlow_Sprint_Planner.xlsx
+++ b/SmartFlow_Sprint_Planner.xlsx
@@ -1143,7 +1143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N35"/>
+  <dimension ref="A1:N39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2389,7 +2389,7 @@
         <v>2.517</v>
       </c>
       <c r="F23" s="29" t="n">
-        <v>1.888</v>
+        <v>2.203</v>
       </c>
       <c r="G23" s="38" t="inlineStr">
         <is>
@@ -3149,6 +3149,10 @@
         <v/>
       </c>
     </row>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <autoFilter ref="A4:L34"/>
   <mergeCells count="1">
@@ -3698,7 +3702,7 @@
       </c>
       <c r="F14" s="41" t="inlineStr">
         <is>
-          <t>Close the remaining Maintenance Scheduler API subtasks. DEV-01/02/03 verified working; TEST-01 and FIX-01 closed by fixing two defects found while testing: the KM range was not ordered (a job from Km 40 to Km 10 saved cleanly, giving every consumer a negative span), and DELETE ignored rowCount so a missing id answered 200 "Deleted" and wrote an audit entry for a deletion that never happened. STILL OPEN: UAT-01 needs real maintenance coordinators - not something that can be closed from the code.</t>
+          <t>Close the remaining Maintenance Scheduler API subtasks. DONE: DEV-01/02/03 verified; TEST-01 and FIX-01 closed by fixing two defects found while testing - the KM range was not ordered (Km 40 to Km 10 saved cleanly, giving every consumer a negative span), and DELETE ignored rowCount so a missing id answered 200 "Deleted" and wrote an audit entry for a deletion that never happened. MAINT is now 7 of 8 subtasks (2.203 of 2.517). STILL OPEN - UAT-01: the interface must be evaluated by maintenance coordinators who can confirm they can plan and organise roadwork with it. That needs real evaluators, not code. ALSO: the existing "Toll Booth Repair" row is entered as Km 76.25 to 73.23 (reversed) and is in progress - correct it by hand; the new validation stops another but does not repair that one.</t>
         </is>
       </c>
       <c r="G14" s="41" t="inlineStr">
@@ -3708,7 +3712,7 @@
       </c>
       <c r="H14" s="42" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="I14" s="70" t="inlineStr">

</xml_diff>